<commit_message>
chore(weekly-sync): auto-pull through 2026-07-12
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Tonor/business_report_week28.xlsx
+++ b/data/ams_weekly_data/Tonor/business_report_week28.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,117 +417,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>(Parent) ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>(Child) ASIN</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Sessions - Total</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Sessions - Total - B2B</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Session Percentage - Total</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Session Percentage - Total - B2B</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Page Views - Total</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Page Views - Total - B2B</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Page Views Percentage - Total</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Page Views Percentage - Total - B2B</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Featured Offer Percentage</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Featured Offer Percentage - B2B</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>units_ordered</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Units Ordered - B2B</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Unit Session Percentage</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Unit Session Percentage - B2B</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>ordered_product_sales</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Ordered Product Sales - B2B</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Total Order Items</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Total Order Items - B2B</t>
         </is>
@@ -614,7 +602,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>53868.48</v>
+        <v>54156.62</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -764,7 +752,7 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
@@ -776,7 +764,7 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>49604.24000000001</v>
+        <v>51891.52</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -922,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
@@ -934,7 +922,7 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>9910.16</v>
+        <v>11604.22</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -1323,7 +1311,7 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
@@ -1335,7 +1323,7 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>29879.67</v>
+        <v>37504.26</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1967,7 +1955,7 @@
         <v>0</v>
       </c>
       <c r="P19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q19" t="n">
         <v>0</v>
@@ -1979,7 +1967,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>6183.91</v>
+        <v>8301.709999999999</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -2129,7 +2117,7 @@
         <v>0</v>
       </c>
       <c r="P21" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="Q21" t="n">
         <v>0</v>
@@ -2141,7 +2129,7 @@
         <v>0</v>
       </c>
       <c r="T21" t="n">
-        <v>22991.52</v>
+        <v>26549.14</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -2453,7 +2441,7 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q25" t="n">
         <v>0</v>
@@ -2465,7 +2453,7 @@
         <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>5421.19</v>
+        <v>7284.75</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2534,7 +2522,7 @@
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="Q26" t="n">
         <v>0</v>
@@ -2546,7 +2534,7 @@
         <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>29309.3</v>
+        <v>34391.51</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>

</xml_diff>